<commit_message>
Assets: Neue Gefahrstoffverzeichnis-Mustervorlage als Download.
Aktualisierte XLSX und Download-Dateiname Gefahrstoffverzeichnis-Mustervorlage.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/downloads/gefahrstoffverzeichnis-vorlage.xlsx
+++ b/downloads/gefahrstoffverzeichnis-vorlage.xlsx
@@ -21,13 +21,7 @@
     <t>Betrieb:</t>
   </si>
   <si>
-    <t>Arbeitsbereich:</t>
-  </si>
-  <si>
     <t>Excel-Chaos beim Gefahrstoffverzeichnis? Schluss mit manuellem Abtippen!</t>
-  </si>
-  <si>
-    <t>Erstellt/Aktualisiert:</t>
   </si>
   <si>
     <r>
@@ -49,7 +43,8 @@
         <sz val="13.0"/>
         <u/>
       </rPr>
-      <t>www.gefahrstoff-qr.de</t>
+      <t xml:space="preserve">www.gefahrstoff-qr.de
+</t>
     </r>
     <r>
       <rPr>
@@ -91,6 +86,12 @@
   </si>
   <si>
     <t>am:</t>
+  </si>
+  <si>
+    <t>Erstellt/Aktualisiert:</t>
+  </si>
+  <si>
+    <t>Arbeitsbereich:</t>
   </si>
   <si>
     <t>Einstufung EG</t>
@@ -196,13 +197,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <sz val="14.0"/>
@@ -389,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -408,7 +409,10 @@
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -721,7 +725,7 @@
     <col customWidth="1" min="3" max="3" width="16.5"/>
     <col customWidth="1" min="4" max="6" width="17.38"/>
     <col customWidth="1" min="7" max="7" width="10.0"/>
-    <col customWidth="1" min="8" max="8" width="44.63"/>
+    <col customWidth="1" min="8" max="8" width="0.38"/>
     <col customWidth="1" min="9" max="9" width="14.63"/>
     <col customWidth="1" min="10" max="10" width="15.25"/>
     <col customWidth="1" min="11" max="13" width="10.0"/>
@@ -749,260 +753,261 @@
       <c r="I2" s="4"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="E3" s="5" t="s">
-        <v>3</v>
       </c>
       <c r="I3" s="4"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="12.75" customHeight="1">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="7" t="s">
+    </row>
+    <row r="6" ht="12.75" customHeight="1">
+      <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" ht="12.75" customHeight="1">
-      <c r="A5" s="6" t="s">
+    <row r="7" ht="12.75" customHeight="1">
+      <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" ht="12.75" customHeight="1">
-      <c r="A6" s="6" t="s">
+    <row r="8" ht="12.75" customHeight="1">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" ht="12.75" customHeight="1"/>
-    <row r="8" ht="12.75" customHeight="1"/>
     <row r="9" ht="18.0" customHeight="1">
-      <c r="C9" s="8"/>
+      <c r="C9" s="9"/>
     </row>
     <row r="10" ht="12.75" customHeight="1"/>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" s="9"/>
+      <c r="A11" s="10"/>
     </row>
     <row r="12" ht="12.75" customHeight="1"/>
     <row r="13" ht="12.75" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" ht="36.0" customHeight="1">
-      <c r="A14" s="11"/>
-      <c r="F14" s="12" t="s">
+      <c r="A14" s="12"/>
+      <c r="F14" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" ht="25.5" customHeight="1">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="H15" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="17" t="s">
+      <c r="J15" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="17" t="s">
+      <c r="K15" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="17" t="s">
+      <c r="L15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="M15" s="14" t="s">
+      <c r="M15" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="14" t="s">
+      <c r="N15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="O15" s="14" t="s">
+      <c r="O15" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="P15" s="18" t="s">
+      <c r="P15" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="Q15" s="19" t="s">
+      <c r="Q15" s="20" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="24"/>
-      <c r="Q16" s="20"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="21"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="21"/>
     </row>
     <row r="17" ht="63.75" customHeight="1">
-      <c r="A17" s="25"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="30"/>
-      <c r="P17" s="31"/>
-      <c r="Q17" s="27"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="31"/>
+      <c r="P17" s="32"/>
+      <c r="Q17" s="28"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="32"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="28"/>
-      <c r="N18" s="28"/>
-      <c r="O18" s="28"/>
-      <c r="P18" s="28"/>
-      <c r="Q18" s="28"/>
+      <c r="A18" s="33"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="29"/>
+      <c r="N18" s="29"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="29"/>
+      <c r="Q18" s="29"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="25"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
-      <c r="O19" s="28"/>
-      <c r="P19" s="28"/>
-      <c r="Q19" s="28"/>
+      <c r="A19" s="26"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
+      <c r="L19" s="29"/>
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="29"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="32"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="28"/>
+      <c r="A20" s="33"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="29"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="25"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28"/>
-      <c r="P21" s="28"/>
-      <c r="Q21" s="28"/>
+      <c r="A21" s="26"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="29"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="29"/>
+      <c r="Q21" s="29"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" s="32"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="28"/>
-      <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28"/>
-      <c r="P22" s="28"/>
-      <c r="Q22" s="28"/>
+      <c r="A22" s="33"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="29"/>
     </row>
     <row r="23" ht="12.75" customHeight="1">
-      <c r="A23" s="25"/>
+      <c r="A23" s="26"/>
     </row>
     <row r="24" ht="12.75" customHeight="1">
-      <c r="A24" s="32"/>
+      <c r="A24" s="33"/>
     </row>
     <row r="25" ht="12.75" customHeight="1">
-      <c r="A25" s="25"/>
+      <c r="A25" s="26"/>
     </row>
     <row r="26" ht="12.75" customHeight="1">
-      <c r="A26" s="32"/>
+      <c r="A26" s="33"/>
     </row>
     <row r="27" ht="12.75" customHeight="1">
-      <c r="A27" s="25"/>
+      <c r="A27" s="26"/>
     </row>
     <row r="28" ht="12.75" customHeight="1"/>
     <row r="29" ht="12.75" customHeight="1"/>
@@ -1991,11 +1996,11 @@
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="Q15:Q16"/>
     <mergeCell ref="I14:L14"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E4"/>
+    <hyperlink r:id="rId1" ref="A4"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>